<commit_message>
SWHC041 Post Processing Updates
Completed Post Processing for SWHC041. Updated Hvac-zone.pxt to include a minimum airflow requirement to resolve EnergyPlus run errors. Updated Normunits to allow "Each" for every Com bldg type.
</commit_message>
<xml_diff>
--- a/scripts/data transformation/Normunits.xlsx
+++ b/scripts/data transformation/Normunits.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\YLIAN\Documents\DEER_github_apr26\DEER-Prototypes-EnergyPlus\scripts\data transformation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DEER-Prototypes-EnergyPlus-TRC_HVAC\scripts\data transformation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F97F49B3-EC2C-4E4A-B881-009059119872}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7E3BBB8-39B7-49B3-8530-8848FD197A52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3372" yWindow="1320" windowWidth="17280" windowHeight="8988" xr2:uid="{527A75FC-5BC9-4372-9120-09678A46B600}"/>
+    <workbookView xWindow="-28920" yWindow="-15" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{527A75FC-5BC9-4372-9120-09678A46B600}"/>
   </bookViews>
   <sheets>
     <sheet name="DMo" sheetId="1" r:id="rId1"/>
@@ -77,7 +77,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="919" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="997" uniqueCount="84">
   <si>
     <t>Normunit</t>
   </si>
@@ -326,6 +326,9 @@
   </si>
   <si>
     <t>6/11/26: Placeholder value, please update for windows</t>
+  </si>
+  <si>
+    <t>added 7/16/2026 to accommodate Normunit = Each for all Com Bldg types</t>
   </si>
 </sst>
 </file>
@@ -711,13 +714,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2593147D-FBCE-4A43-B94C-18CB04EC4F0B}">
   <dimension ref="A1:F8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -737,7 +740,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -748,7 +751,7 @@
         <v>2480</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>20</v>
       </c>
@@ -762,7 +765,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>20</v>
       </c>
@@ -776,7 +779,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>20</v>
       </c>
@@ -793,7 +796,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>30</v>
       </c>
@@ -808,7 +811,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>68</v>
       </c>
@@ -825,7 +828,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>65</v>
       </c>
@@ -845,13 +848,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C9AEBA2-4873-4E93-88D1-6559970F8CAA}">
   <dimension ref="A1:F55"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -871,7 +874,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -882,7 +885,7 @@
         <v>24580</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>20</v>
       </c>
@@ -896,7 +899,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>20</v>
       </c>
@@ -910,7 +913,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>20</v>
       </c>
@@ -927,7 +930,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>68</v>
       </c>
@@ -944,7 +947,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>68</v>
       </c>
@@ -961,7 +964,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>68</v>
       </c>
@@ -978,7 +981,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>68</v>
       </c>
@@ -995,7 +998,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>68</v>
       </c>
@@ -1012,7 +1015,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>68</v>
       </c>
@@ -1029,7 +1032,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>68</v>
       </c>
@@ -1046,7 +1049,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>68</v>
       </c>
@@ -1063,7 +1066,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>68</v>
       </c>
@@ -1080,7 +1083,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>68</v>
       </c>
@@ -1097,7 +1100,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>68</v>
       </c>
@@ -1114,7 +1117,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>68</v>
       </c>
@@ -1131,7 +1134,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>68</v>
       </c>
@@ -1148,7 +1151,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>68</v>
       </c>
@@ -1165,7 +1168,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>68</v>
       </c>
@@ -1182,7 +1185,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>68</v>
       </c>
@@ -1199,7 +1202,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>68</v>
       </c>
@@ -1216,7 +1219,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>68</v>
       </c>
@@ -1233,7 +1236,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>68</v>
       </c>
@@ -1250,7 +1253,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>68</v>
       </c>
@@ -1267,7 +1270,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>68</v>
       </c>
@@ -1284,7 +1287,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>68</v>
       </c>
@@ -1301,7 +1304,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>68</v>
       </c>
@@ -1318,7 +1321,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>68</v>
       </c>
@@ -1335,7 +1338,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>68</v>
       </c>
@@ -1352,7 +1355,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>68</v>
       </c>
@@ -1369,7 +1372,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>68</v>
       </c>
@@ -1386,7 +1389,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>68</v>
       </c>
@@ -1403,7 +1406,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>68</v>
       </c>
@@ -1420,7 +1423,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>68</v>
       </c>
@@ -1437,7 +1440,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>68</v>
       </c>
@@ -1454,7 +1457,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>68</v>
       </c>
@@ -1471,7 +1474,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>30</v>
       </c>
@@ -1486,7 +1489,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>68</v>
       </c>
@@ -1503,7 +1506,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>68</v>
       </c>
@@ -1520,7 +1523,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>68</v>
       </c>
@@ -1537,7 +1540,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>68</v>
       </c>
@@ -1554,7 +1557,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>68</v>
       </c>
@@ -1571,7 +1574,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>68</v>
       </c>
@@ -1588,7 +1591,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>68</v>
       </c>
@@ -1605,7 +1608,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>68</v>
       </c>
@@ -1622,7 +1625,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>68</v>
       </c>
@@ -1639,7 +1642,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>68</v>
       </c>
@@ -1656,7 +1659,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>68</v>
       </c>
@@ -1673,7 +1676,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>68</v>
       </c>
@@ -1690,7 +1693,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>68</v>
       </c>
@@ -1707,7 +1710,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>68</v>
       </c>
@@ -1724,7 +1727,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>68</v>
       </c>
@@ -1741,7 +1744,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>68</v>
       </c>
@@ -1758,7 +1761,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>65</v>
       </c>
@@ -1778,14 +1781,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D254DEF8-D70B-44A9-90B7-19C720405132}">
   <dimension ref="A1:F116"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.21875" customWidth="1"/>
-    <col min="4" max="4" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.28515625" customWidth="1"/>
+    <col min="4" max="4" width="14.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1805,7 +1808,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -1816,7 +1819,7 @@
         <v>4320</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -1827,7 +1830,7 @@
         <v>4320</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -1838,7 +1841,7 @@
         <v>4320</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>1</v>
       </c>
@@ -1849,7 +1852,7 @@
         <v>4320</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>1</v>
       </c>
@@ -1860,7 +1863,7 @@
         <v>4320</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>1</v>
       </c>
@@ -1871,7 +1874,7 @@
         <v>4500</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>1</v>
       </c>
@@ -1882,7 +1885,7 @@
         <v>4500</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>1</v>
       </c>
@@ -1893,7 +1896,7 @@
         <v>4500</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>1</v>
       </c>
@@ -1904,7 +1907,7 @@
         <v>3850</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>1</v>
       </c>
@@ -1915,7 +1918,7 @@
         <v>4140</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>1</v>
       </c>
@@ -1926,7 +1929,7 @@
         <v>3570</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>1</v>
       </c>
@@ -1937,7 +1940,7 @@
         <v>3570</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>1</v>
       </c>
@@ -1948,7 +1951,7 @@
         <v>3570</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>1</v>
       </c>
@@ -1959,7 +1962,7 @@
         <v>3250</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>1</v>
       </c>
@@ -1970,7 +1973,7 @@
         <v>3250</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>1</v>
       </c>
@@ -1981,7 +1984,7 @@
         <v>3800</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>20</v>
       </c>
@@ -1995,7 +1998,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>20</v>
       </c>
@@ -2009,7 +2012,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>20</v>
       </c>
@@ -2023,7 +2026,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -2037,7 +2040,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>20</v>
       </c>
@@ -2051,7 +2054,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>20</v>
       </c>
@@ -2065,7 +2068,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>20</v>
       </c>
@@ -2079,7 +2082,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>20</v>
       </c>
@@ -2093,7 +2096,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>20</v>
       </c>
@@ -2107,7 +2110,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>20</v>
       </c>
@@ -2121,7 +2124,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>20</v>
       </c>
@@ -2135,7 +2138,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>20</v>
       </c>
@@ -2149,7 +2152,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>20</v>
       </c>
@@ -2163,7 +2166,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>20</v>
       </c>
@@ -2177,7 +2180,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>20</v>
       </c>
@@ -2191,7 +2194,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>20</v>
       </c>
@@ -2205,7 +2208,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>20</v>
       </c>
@@ -2219,7 +2222,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>20</v>
       </c>
@@ -2233,7 +2236,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>20</v>
       </c>
@@ -2247,7 +2250,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>20</v>
       </c>
@@ -2261,7 +2264,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>20</v>
       </c>
@@ -2275,7 +2278,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>20</v>
       </c>
@@ -2289,7 +2292,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>20</v>
       </c>
@@ -2303,7 +2306,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>20</v>
       </c>
@@ -2317,7 +2320,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>20</v>
       </c>
@@ -2331,7 +2334,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>20</v>
       </c>
@@ -2345,7 +2348,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>20</v>
       </c>
@@ -2359,7 +2362,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>20</v>
       </c>
@@ -2373,7 +2376,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>20</v>
       </c>
@@ -2387,7 +2390,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>20</v>
       </c>
@@ -2401,7 +2404,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>20</v>
       </c>
@@ -2415,7 +2418,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>20</v>
       </c>
@@ -2429,7 +2432,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>68</v>
       </c>
@@ -2446,7 +2449,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>68</v>
       </c>
@@ -2463,7 +2466,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>68</v>
       </c>
@@ -2480,7 +2483,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>68</v>
       </c>
@@ -2497,7 +2500,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>68</v>
       </c>
@@ -2514,7 +2517,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>68</v>
       </c>
@@ -2531,7 +2534,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>68</v>
       </c>
@@ -2548,7 +2551,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>68</v>
       </c>
@@ -2565,7 +2568,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>68</v>
       </c>
@@ -2582,7 +2585,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>68</v>
       </c>
@@ -2599,7 +2602,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>68</v>
       </c>
@@ -2616,7 +2619,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>68</v>
       </c>
@@ -2633,7 +2636,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>68</v>
       </c>
@@ -2650,7 +2653,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>68</v>
       </c>
@@ -2667,7 +2670,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>68</v>
       </c>
@@ -2684,7 +2687,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>68</v>
       </c>
@@ -2701,7 +2704,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>68</v>
       </c>
@@ -2718,7 +2721,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>68</v>
       </c>
@@ -2735,7 +2738,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>68</v>
       </c>
@@ -2752,7 +2755,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>68</v>
       </c>
@@ -2769,7 +2772,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>68</v>
       </c>
@@ -2786,7 +2789,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>68</v>
       </c>
@@ -2803,7 +2806,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>68</v>
       </c>
@@ -2820,7 +2823,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>68</v>
       </c>
@@ -2837,7 +2840,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>68</v>
       </c>
@@ -2854,7 +2857,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>68</v>
       </c>
@@ -2871,7 +2874,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>68</v>
       </c>
@@ -2888,7 +2891,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>68</v>
       </c>
@@ -2905,7 +2908,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>68</v>
       </c>
@@ -2922,7 +2925,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>68</v>
       </c>
@@ -2939,7 +2942,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>68</v>
       </c>
@@ -2956,7 +2959,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>68</v>
       </c>
@@ -2973,7 +2976,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>28</v>
       </c>
@@ -2987,7 +2990,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>30</v>
       </c>
@@ -3002,7 +3005,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>65</v>
       </c>
@@ -3013,7 +3016,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>68</v>
       </c>
@@ -3030,7 +3033,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>68</v>
       </c>
@@ -3047,7 +3050,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>68</v>
       </c>
@@ -3064,7 +3067,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>68</v>
       </c>
@@ -3081,7 +3084,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>68</v>
       </c>
@@ -3098,7 +3101,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>68</v>
       </c>
@@ -3115,7 +3118,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>68</v>
       </c>
@@ -3132,7 +3135,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>68</v>
       </c>
@@ -3149,7 +3152,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>68</v>
       </c>
@@ -3166,7 +3169,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>68</v>
       </c>
@@ -3183,7 +3186,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>68</v>
       </c>
@@ -3200,7 +3203,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>68</v>
       </c>
@@ -3217,7 +3220,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>68</v>
       </c>
@@ -3234,7 +3237,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>68</v>
       </c>
@@ -3251,7 +3254,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>68</v>
       </c>
@@ -3268,7 +3271,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>68</v>
       </c>
@@ -3285,7 +3288,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>20</v>
       </c>
@@ -3302,7 +3305,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>20</v>
       </c>
@@ -3319,7 +3322,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>20</v>
       </c>
@@ -3336,7 +3339,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>20</v>
       </c>
@@ -3353,7 +3356,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>20</v>
       </c>
@@ -3370,7 +3373,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>20</v>
       </c>
@@ -3387,7 +3390,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>20</v>
       </c>
@@ -3404,7 +3407,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>20</v>
       </c>
@@ -3421,7 +3424,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>20</v>
       </c>
@@ -3438,7 +3441,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>20</v>
       </c>
@@ -3455,7 +3458,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>20</v>
       </c>
@@ -3472,7 +3475,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>20</v>
       </c>
@@ -3489,7 +3492,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>20</v>
       </c>
@@ -3506,7 +3509,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>20</v>
       </c>
@@ -3523,7 +3526,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>20</v>
       </c>
@@ -3540,7 +3543,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>20</v>
       </c>
@@ -3567,18 +3570,18 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F653D6A-2407-4550-AC1C-A4556A4DAC9A}">
-  <dimension ref="A1:I88"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:I114"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="22.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.33203125" customWidth="1"/>
-    <col min="5" max="5" width="20.44140625" customWidth="1"/>
-    <col min="6" max="6" width="11.21875" customWidth="1"/>
+    <col min="3" max="3" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.28515625" customWidth="1"/>
+    <col min="5" max="5" width="20.42578125" customWidth="1"/>
+    <col min="6" max="6" width="11.28515625" customWidth="1"/>
     <col min="7" max="7" width="15" customWidth="1"/>
-    <col min="9" max="9" width="13.6640625" customWidth="1"/>
+    <col min="9" max="9" width="13.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>33</v>
       </c>
@@ -3607,7 +3610,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>34</v>
       </c>
@@ -3626,7 +3629,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>35</v>
       </c>
@@ -3645,7 +3648,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>36</v>
       </c>
@@ -3664,7 +3667,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>37</v>
       </c>
@@ -3683,7 +3686,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>38</v>
       </c>
@@ -3702,7 +3705,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>39</v>
       </c>
@@ -3721,7 +3724,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>57</v>
       </c>
@@ -3740,7 +3743,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>58</v>
       </c>
@@ -3759,7 +3762,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>40</v>
       </c>
@@ -3778,7 +3781,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>41</v>
       </c>
@@ -3797,7 +3800,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>59</v>
       </c>
@@ -3816,7 +3819,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>42</v>
       </c>
@@ -3835,7 +3838,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>43</v>
       </c>
@@ -3854,7 +3857,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>44</v>
       </c>
@@ -3873,7 +3876,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>45</v>
       </c>
@@ -3892,7 +3895,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>46</v>
       </c>
@@ -3911,7 +3914,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>47</v>
       </c>
@@ -3930,7 +3933,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>60</v>
       </c>
@@ -3949,7 +3952,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>48</v>
       </c>
@@ -3968,7 +3971,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>49</v>
       </c>
@@ -3987,7 +3990,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>50</v>
       </c>
@@ -4006,7 +4009,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>51</v>
       </c>
@@ -4025,7 +4028,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>52</v>
       </c>
@@ -4044,7 +4047,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>53</v>
       </c>
@@ -4063,7 +4066,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>61</v>
       </c>
@@ -4082,7 +4085,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>62</v>
       </c>
@@ -4101,7 +4104,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>3</v>
       </c>
@@ -4115,768 +4118,1132 @@
         <v>66</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>34</v>
       </c>
       <c r="C29" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F29">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I29" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>35</v>
       </c>
       <c r="C30" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F30">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I30" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>36</v>
       </c>
       <c r="C31" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F31">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I31" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>37</v>
       </c>
       <c r="C32" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F32">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I32" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>38</v>
       </c>
       <c r="C33" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F33">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I33" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>39</v>
       </c>
       <c r="C34" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F34">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I34" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>57</v>
       </c>
       <c r="C35" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F35">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I35" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>58</v>
       </c>
       <c r="C36" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F36">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I36" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>40</v>
       </c>
       <c r="C37" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F37">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I37" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>41</v>
       </c>
       <c r="C38" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F38">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I38" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>59</v>
       </c>
       <c r="C39" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F39">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I39" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>42</v>
       </c>
       <c r="C40" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F40">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I40" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>43</v>
       </c>
       <c r="C41" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F41">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I41" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>44</v>
       </c>
       <c r="C42" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F42">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I42" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>45</v>
       </c>
       <c r="C43" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F43">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I43" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>46</v>
       </c>
       <c r="C44" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F44">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I44" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>47</v>
       </c>
       <c r="C45" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F45">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I45" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>60</v>
       </c>
       <c r="C46" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F46">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I46" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>48</v>
       </c>
       <c r="C47" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F47">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I47" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>49</v>
       </c>
       <c r="C48" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F48">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I48" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>50</v>
       </c>
       <c r="C49" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F49">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I49" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.3">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>51</v>
       </c>
       <c r="C50" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F50">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I50" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.3">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>52</v>
       </c>
       <c r="C51" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F51">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I51" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.3">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>53</v>
       </c>
       <c r="C52" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F52">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I52" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.3">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>61</v>
       </c>
       <c r="C53" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F53">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I53" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.3">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>62</v>
       </c>
       <c r="C54" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F54">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I54" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.3">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>34</v>
       </c>
       <c r="C55" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F55">
-        <v>60</v>
+        <v>10</v>
       </c>
       <c r="I55" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.3">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>35</v>
       </c>
       <c r="C56" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F56">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+      <c r="I56" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>36</v>
       </c>
       <c r="C57" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F57">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+      <c r="I57" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>37</v>
       </c>
       <c r="C58" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F58">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+      <c r="I58" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>38</v>
       </c>
       <c r="C59" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F59">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+      <c r="I59" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>39</v>
       </c>
       <c r="C60" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F60">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+      <c r="I60" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>57</v>
       </c>
       <c r="C61" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F61">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+      <c r="I61" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>58</v>
       </c>
       <c r="C62" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F62">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+      <c r="I62" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>40</v>
       </c>
       <c r="C63" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F63">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+      <c r="I63" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>41</v>
       </c>
       <c r="C64" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F64">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+      <c r="I64" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>59</v>
       </c>
       <c r="C65" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F65">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+      <c r="I65" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>42</v>
       </c>
       <c r="C66" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F66">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+      <c r="I66" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>43</v>
       </c>
       <c r="C67" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F67">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+      <c r="I67" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>44</v>
       </c>
       <c r="C68" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F68">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+      <c r="I68" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>45</v>
       </c>
       <c r="C69" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F69">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+      <c r="I69" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>46</v>
       </c>
       <c r="C70" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F70">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+      <c r="I70" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>47</v>
       </c>
       <c r="C71" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F71">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+      <c r="I71" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>60</v>
       </c>
       <c r="C72" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F72">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+      <c r="I72" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="73" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>48</v>
       </c>
       <c r="C73" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F73">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+      <c r="I73" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="74" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>49</v>
       </c>
       <c r="C74" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F74">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+      <c r="I74" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="75" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>50</v>
       </c>
       <c r="C75" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F75">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+      <c r="I75" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="76" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>51</v>
       </c>
       <c r="C76" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F76">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+      <c r="I76" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="77" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>52</v>
       </c>
       <c r="C77" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F77">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+      <c r="I77" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="78" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>53</v>
       </c>
       <c r="C78" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F78">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+      <c r="I78" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="79" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>61</v>
       </c>
       <c r="C79" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F79">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+      <c r="I79" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="80" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>62</v>
       </c>
       <c r="C80" t="s">
+        <v>68</v>
+      </c>
+      <c r="F80">
+        <v>10</v>
+      </c>
+      <c r="I80" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="81" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>34</v>
+      </c>
+      <c r="C81" t="s">
         <v>69</v>
       </c>
-      <c r="F80">
+      <c r="F81">
         <v>60</v>
       </c>
-    </row>
-    <row r="81" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A81" t="s">
+      <c r="I81" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="82" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>35</v>
+      </c>
+      <c r="C82" t="s">
+        <v>69</v>
+      </c>
+      <c r="F82">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="83" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>36</v>
+      </c>
+      <c r="C83" t="s">
+        <v>69</v>
+      </c>
+      <c r="F83">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="84" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>37</v>
+      </c>
+      <c r="C84" t="s">
+        <v>69</v>
+      </c>
+      <c r="F84">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="85" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>38</v>
+      </c>
+      <c r="C85" t="s">
+        <v>69</v>
+      </c>
+      <c r="F85">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="86" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>39</v>
+      </c>
+      <c r="C86" t="s">
+        <v>69</v>
+      </c>
+      <c r="F86">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="87" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>57</v>
+      </c>
+      <c r="C87" t="s">
+        <v>69</v>
+      </c>
+      <c r="F87">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="88" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
         <v>58</v>
       </c>
-      <c r="C81" t="s">
+      <c r="C88" t="s">
+        <v>69</v>
+      </c>
+      <c r="F88">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="89" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>40</v>
+      </c>
+      <c r="C89" t="s">
+        <v>69</v>
+      </c>
+      <c r="F89">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="90" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>41</v>
+      </c>
+      <c r="C90" t="s">
+        <v>69</v>
+      </c>
+      <c r="F90">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="91" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>59</v>
+      </c>
+      <c r="C91" t="s">
+        <v>69</v>
+      </c>
+      <c r="F91">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="92" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>42</v>
+      </c>
+      <c r="C92" t="s">
+        <v>69</v>
+      </c>
+      <c r="F92">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="93" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>43</v>
+      </c>
+      <c r="C93" t="s">
+        <v>69</v>
+      </c>
+      <c r="F93">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="94" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>44</v>
+      </c>
+      <c r="C94" t="s">
+        <v>69</v>
+      </c>
+      <c r="F94">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="95" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>45</v>
+      </c>
+      <c r="C95" t="s">
+        <v>69</v>
+      </c>
+      <c r="F95">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="96" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>46</v>
+      </c>
+      <c r="C96" t="s">
+        <v>69</v>
+      </c>
+      <c r="F96">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="97" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>47</v>
+      </c>
+      <c r="C97" t="s">
+        <v>69</v>
+      </c>
+      <c r="F97">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="98" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>60</v>
+      </c>
+      <c r="C98" t="s">
+        <v>69</v>
+      </c>
+      <c r="F98">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="99" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>48</v>
+      </c>
+      <c r="C99" t="s">
+        <v>69</v>
+      </c>
+      <c r="F99">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="100" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>49</v>
+      </c>
+      <c r="C100" t="s">
+        <v>69</v>
+      </c>
+      <c r="F100">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="101" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>50</v>
+      </c>
+      <c r="C101" t="s">
+        <v>69</v>
+      </c>
+      <c r="F101">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="102" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>51</v>
+      </c>
+      <c r="C102" t="s">
+        <v>69</v>
+      </c>
+      <c r="F102">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="103" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>52</v>
+      </c>
+      <c r="C103" t="s">
+        <v>69</v>
+      </c>
+      <c r="F103">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="104" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>53</v>
+      </c>
+      <c r="C104" t="s">
+        <v>69</v>
+      </c>
+      <c r="F104">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="105" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>61</v>
+      </c>
+      <c r="C105" t="s">
+        <v>69</v>
+      </c>
+      <c r="F105">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="106" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>62</v>
+      </c>
+      <c r="C106" t="s">
+        <v>69</v>
+      </c>
+      <c r="F106">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="107" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>58</v>
+      </c>
+      <c r="C107" t="s">
         <v>72</v>
       </c>
-      <c r="F81">
+      <c r="F107">
         <v>12</v>
       </c>
-      <c r="I81" t="s">
+      <c r="I107" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="82" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A82" t="s">
+    <row r="108" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
         <v>58</v>
       </c>
-      <c r="C82" t="s">
+      <c r="C108" t="s">
         <v>73</v>
       </c>
-      <c r="F82">
+      <c r="F108">
         <v>12</v>
       </c>
-      <c r="I82" t="s">
+      <c r="I108" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="83" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A83" t="s">
+    <row r="109" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
         <v>3</v>
       </c>
-      <c r="B83" t="s">
+      <c r="B109" t="s">
         <v>4</v>
       </c>
-      <c r="C83" t="s">
+      <c r="C109" t="s">
         <v>74</v>
       </c>
-      <c r="F83">
+      <c r="F109">
         <v>10</v>
       </c>
-      <c r="I83" t="s">
+      <c r="I109" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="84" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A84" t="s">
+    <row r="110" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
         <v>3</v>
       </c>
-      <c r="B84" t="s">
+      <c r="B110" t="s">
         <v>5</v>
       </c>
-      <c r="C84" t="s">
+      <c r="C110" t="s">
         <v>74</v>
       </c>
-      <c r="F84">
+      <c r="F110">
         <v>20</v>
       </c>
-      <c r="I84" t="s">
+      <c r="I110" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="85" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A85" t="s">
+    <row r="111" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
         <v>3</v>
       </c>
-      <c r="B85" t="s">
+      <c r="B111" t="s">
         <v>6</v>
       </c>
-      <c r="C85" t="s">
+      <c r="C111" t="s">
         <v>74</v>
       </c>
-      <c r="F85">
+      <c r="F111">
         <v>30</v>
       </c>
-      <c r="I85" t="s">
+      <c r="I111" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="86" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A86" t="s">
+    <row r="112" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
         <v>34</v>
       </c>
-      <c r="C86" t="s">
+      <c r="C112" t="s">
         <v>77</v>
       </c>
-      <c r="I86" t="s">
+      <c r="I112" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="87" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A87" t="s">
+    <row r="113" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
         <v>35</v>
       </c>
-      <c r="C87" t="s">
+      <c r="C113" t="s">
         <v>77</v>
       </c>
-      <c r="I87" t="s">
+      <c r="I113" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="88" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A88" t="s">
+    <row r="114" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
         <v>36</v>
       </c>
-      <c r="C88" t="s">
+      <c r="C114" t="s">
         <v>77</v>
       </c>
-      <c r="I88" t="s">
+      <c r="I114" t="s">
         <v>75</v>
       </c>
     </row>
@@ -4889,14 +5256,14 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{494C52AA-17FA-4976-ACAF-0C5241107ABB}">
   <dimension ref="A1:D27"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>33</v>
       </c>
@@ -4910,7 +5277,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>34</v>
       </c>
@@ -4925,7 +5292,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>35</v>
       </c>
@@ -4937,7 +5304,7 @@
         <v>284192.63738854404</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>36</v>
       </c>
@@ -4949,7 +5316,7 @@
         <v>40745.491149952002</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>37</v>
       </c>
@@ -4961,7 +5328,7 @@
         <v>2883.5439570559997</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>38</v>
       </c>
@@ -4973,7 +5340,7 @@
         <v>74402.301466880002</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>39</v>
       </c>
@@ -4985,7 +5352,7 @@
         <v>857786.46076908801</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>57</v>
       </c>
@@ -4997,7 +5364,7 @@
         <v>3599.9898332799999</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>58</v>
       </c>
@@ -5009,7 +5376,7 @@
         <v>49996.964499647998</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>40</v>
       </c>
@@ -5021,7 +5388,7 @@
         <v>494055.84498361603</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>41</v>
       </c>
@@ -5033,7 +5400,7 @@
         <v>137116.71846502399</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>59</v>
       </c>
@@ -5045,7 +5412,7 @@
         <v>9999.9956789120006</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>42</v>
       </c>
@@ -5057,7 +5424,7 @@
         <v>399947.62219104002</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>43</v>
       </c>
@@ -5069,7 +5436,7 @@
         <v>100014.057511744</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>44</v>
       </c>
@@ -5081,7 +5448,7 @@
         <v>29986.209231424</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>45</v>
       </c>
@@ -5093,7 +5460,7 @@
         <v>110998.73571404802</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>46</v>
       </c>
@@ -5105,7 +5472,7 @@
         <v>349919.98054675205</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>47</v>
       </c>
@@ -5117,7 +5484,7 @@
         <v>20004.619839296</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>60</v>
       </c>
@@ -5129,7 +5496,7 @@
         <v>19999.776079616</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>48</v>
       </c>
@@ -5141,7 +5508,7 @@
         <v>3996.2093751040002</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>49</v>
       </c>
@@ -5153,7 +5520,7 @@
         <v>11205.123087296</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>50</v>
       </c>
@@ -5165,7 +5532,7 @@
         <v>240000.003932992</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>51</v>
       </c>
@@ -5177,7 +5544,7 @@
         <v>130501.54205049601</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>52</v>
       </c>
@@ -5189,7 +5556,7 @@
         <v>16002.597952576001</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>53</v>
       </c>
@@ -5201,7 +5568,7 @@
         <v>499990.41934355197</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>61</v>
       </c>
@@ -5213,7 +5580,7 @@
         <v>499990.41934355197</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>62</v>
       </c>

</xml_diff>